<commit_message>
Comparing mortalities (actuarial table vs model - remove variability)
</commit_message>
<xml_diff>
--- a/2022 Actuarial Life Table.xlsx
+++ b/2022 Actuarial Life Table.xlsx
@@ -8,19 +8,33 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sodamkim/Library/CloudStorage/Box-Box/ATTR-CM_SK/CEA/Microsimulation/Dark Peak Analytics/TRACE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{86D6B109-D197-9340-B0C2-2A9FEF07E516}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6064FC80-04DB-C444-9D3D-5D7B97B6BFF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11580" yWindow="5480" windowWidth="28040" windowHeight="17180" xr2:uid="{49FD46BD-3C6D-9D48-A728-0523D1ADC09C}"/>
+    <workbookView xWindow="22380" yWindow="4000" windowWidth="28040" windowHeight="17180" activeTab="1" xr2:uid="{49FD46BD-3C6D-9D48-A728-0523D1ADC09C}"/>
   </bookViews>
   <sheets>
     <sheet name="2022 Actuarial Life Table" sheetId="1" r:id="rId1"/>
+    <sheet name="Comparing mortalities" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Exact age</t>
   </si>
@@ -41,6 +55,18 @@
   </si>
   <si>
     <t>Female Life expectancy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Actuarial table </t>
+  </si>
+  <si>
+    <t>Actuarial table</t>
+  </si>
+  <si>
+    <t>Gompertz + SD 0</t>
+  </si>
+  <si>
+    <t>Lookuptable + SD 0</t>
   </si>
 </sst>
 </file>
@@ -901,8 +927,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66E35FB3-3F0E-5F4C-BAAB-CFA32CE9AB1F}">
-  <dimension ref="A1:G121"/>
+  <dimension ref="A1:K121"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="27.1640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -2376,7 +2405,7 @@
         <v>22.5</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>63</v>
       </c>
@@ -2399,7 +2428,7 @@
         <v>21.7</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>64</v>
       </c>
@@ -2422,7 +2451,7 @@
         <v>20.9</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>65</v>
       </c>
@@ -2445,7 +2474,7 @@
         <v>20.12</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>66</v>
       </c>
@@ -2468,7 +2497,7 @@
         <v>19.34</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>67</v>
       </c>
@@ -2491,7 +2520,7 @@
         <v>18.559999999999999</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>68</v>
       </c>
@@ -2514,7 +2543,7 @@
         <v>17.79</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>69</v>
       </c>
@@ -2537,7 +2566,7 @@
         <v>17.03</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>70</v>
       </c>
@@ -2560,7 +2589,7 @@
         <v>16.27</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>71</v>
       </c>
@@ -2583,7 +2612,7 @@
         <v>15.53</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>72</v>
       </c>
@@ -2606,7 +2635,7 @@
         <v>14.8</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>73</v>
       </c>
@@ -2629,7 +2658,7 @@
         <v>14.08</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>74</v>
       </c>
@@ -2652,7 +2681,7 @@
         <v>13.37</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>75</v>
       </c>
@@ -2675,7 +2704,7 @@
         <v>12.68</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>76</v>
       </c>
@@ -2697,8 +2726,11 @@
       <c r="G78">
         <v>12</v>
       </c>
-    </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="K78" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>77</v>
       </c>
@@ -2720,8 +2752,20 @@
       <c r="G79">
         <v>11.35</v>
       </c>
-    </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I79">
+        <f>1-B79</f>
+        <v>0.95475900000000002</v>
+      </c>
+      <c r="J79">
+        <f>SQRT(I79)</f>
+        <v>0.97711770017741462</v>
+      </c>
+      <c r="K79">
+        <f>1-J79</f>
+        <v>2.2882299822585384E-2</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>78</v>
       </c>
@@ -2743,8 +2787,20 @@
       <c r="G80">
         <v>10.71</v>
       </c>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I80">
+        <f t="shared" ref="I80:I121" si="0">1-B80</f>
+        <v>0.95020700000000002</v>
+      </c>
+      <c r="J80">
+        <f t="shared" ref="J80:J121" si="1">SQRT(I80)</f>
+        <v>0.97478561745647441</v>
+      </c>
+      <c r="K80">
+        <f t="shared" ref="K80:K121" si="2">1-J80</f>
+        <v>2.5214382543525593E-2</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>79</v>
       </c>
@@ -2766,8 +2822,20 @@
       <c r="G81">
         <v>10.09</v>
       </c>
-    </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I81">
+        <f t="shared" si="0"/>
+        <v>0.94523199999999996</v>
+      </c>
+      <c r="J81">
+        <f t="shared" si="1"/>
+        <v>0.97223042536221826</v>
+      </c>
+      <c r="K81">
+        <f t="shared" si="2"/>
+        <v>2.7769574637781735E-2</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>80</v>
       </c>
@@ -2789,8 +2857,20 @@
       <c r="G82">
         <v>9.49</v>
       </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I82">
+        <f t="shared" si="0"/>
+        <v>0.93933999999999995</v>
+      </c>
+      <c r="J82">
+        <f t="shared" si="1"/>
+        <v>0.96919554270539232</v>
+      </c>
+      <c r="K82">
+        <f t="shared" si="2"/>
+        <v>3.0804457294607679E-2</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>81</v>
       </c>
@@ -2812,8 +2892,20 @@
       <c r="G83">
         <v>8.9</v>
       </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I83">
+        <f t="shared" si="0"/>
+        <v>0.93297300000000005</v>
+      </c>
+      <c r="J83">
+        <f t="shared" si="1"/>
+        <v>0.96590527485877209</v>
+      </c>
+      <c r="K83">
+        <f t="shared" si="2"/>
+        <v>3.4094725141227911E-2</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>82</v>
       </c>
@@ -2835,8 +2927,20 @@
       <c r="G84">
         <v>8.34</v>
       </c>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I84">
+        <f t="shared" si="0"/>
+        <v>0.92600099999999996</v>
+      </c>
+      <c r="J84">
+        <f t="shared" si="1"/>
+        <v>0.96228945749187134</v>
+      </c>
+      <c r="K84">
+        <f t="shared" si="2"/>
+        <v>3.7710542508128664E-2</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>83</v>
       </c>
@@ -2858,8 +2962,20 @@
       <c r="G85">
         <v>7.79</v>
       </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I85">
+        <f t="shared" si="0"/>
+        <v>0.91826300000000005</v>
+      </c>
+      <c r="J85">
+        <f t="shared" si="1"/>
+        <v>0.95826040302205961</v>
+      </c>
+      <c r="K85">
+        <f t="shared" si="2"/>
+        <v>4.1739596977940385E-2</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>84</v>
       </c>
@@ -2881,8 +2997,20 @@
       <c r="G86">
         <v>7.26</v>
       </c>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I86">
+        <f t="shared" si="0"/>
+        <v>0.90954199999999996</v>
+      </c>
+      <c r="J86">
+        <f t="shared" si="1"/>
+        <v>0.95369911397673002</v>
+      </c>
+      <c r="K86">
+        <f t="shared" si="2"/>
+        <v>4.6300886023269983E-2</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>85</v>
       </c>
@@ -2904,8 +3032,20 @@
       <c r="G87">
         <v>6.76</v>
       </c>
-    </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I87">
+        <f t="shared" si="0"/>
+        <v>0.89947500000000002</v>
+      </c>
+      <c r="J87">
+        <f t="shared" si="1"/>
+        <v>0.9484065583914949</v>
+      </c>
+      <c r="K87">
+        <f t="shared" si="2"/>
+        <v>5.1593441608505097E-2</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>86</v>
       </c>
@@ -2927,8 +3067,20 @@
       <c r="G88">
         <v>6.28</v>
       </c>
-    </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I88">
+        <f t="shared" si="0"/>
+        <v>0.88820699999999997</v>
+      </c>
+      <c r="J88">
+        <f t="shared" si="1"/>
+        <v>0.94244734600931424</v>
+      </c>
+      <c r="K88">
+        <f t="shared" si="2"/>
+        <v>5.7552653990685765E-2</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>87</v>
       </c>
@@ -2950,8 +3102,20 @@
       <c r="G89">
         <v>5.83</v>
       </c>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I89">
+        <f t="shared" si="0"/>
+        <v>0.87550600000000001</v>
+      </c>
+      <c r="J89">
+        <f t="shared" si="1"/>
+        <v>0.93568477597960309</v>
+      </c>
+      <c r="K89">
+        <f t="shared" si="2"/>
+        <v>6.4315224020396911E-2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>88</v>
       </c>
@@ -2973,8 +3137,20 @@
       <c r="G90">
         <v>5.4</v>
       </c>
-    </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I90">
+        <f t="shared" si="0"/>
+        <v>0.86160199999999998</v>
+      </c>
+      <c r="J90">
+        <f t="shared" si="1"/>
+        <v>0.92822518819519217</v>
+      </c>
+      <c r="K90">
+        <f t="shared" si="2"/>
+        <v>7.1774811804807825E-2</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>89</v>
       </c>
@@ -2996,8 +3172,20 @@
       <c r="G91">
         <v>5</v>
       </c>
-    </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I91">
+        <f t="shared" si="0"/>
+        <v>0.84679300000000002</v>
+      </c>
+      <c r="J91">
+        <f t="shared" si="1"/>
+        <v>0.92021356216913042</v>
+      </c>
+      <c r="K91">
+        <f t="shared" si="2"/>
+        <v>7.9786437830869583E-2</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>90</v>
       </c>
@@ -3019,8 +3207,20 @@
       <c r="G92">
         <v>4.62</v>
       </c>
-    </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I92">
+        <f t="shared" si="0"/>
+        <v>0.83029600000000003</v>
+      </c>
+      <c r="J92">
+        <f t="shared" si="1"/>
+        <v>0.91120579453820416</v>
+      </c>
+      <c r="K92">
+        <f t="shared" si="2"/>
+        <v>8.8794205461795839E-2</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>91</v>
       </c>
@@ -3042,8 +3242,20 @@
       <c r="G93">
         <v>4.2699999999999996</v>
       </c>
-    </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I93">
+        <f t="shared" si="0"/>
+        <v>0.81203700000000001</v>
+      </c>
+      <c r="J93">
+        <f t="shared" si="1"/>
+        <v>0.90113095607686233</v>
+      </c>
+      <c r="K93">
+        <f t="shared" si="2"/>
+        <v>9.8869043923137667E-2</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>92</v>
       </c>
@@ -3065,8 +3277,20 @@
       <c r="G94">
         <v>3.94</v>
       </c>
-    </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I94">
+        <f t="shared" si="0"/>
+        <v>0.791605</v>
+      </c>
+      <c r="J94">
+        <f t="shared" si="1"/>
+        <v>0.88972186665271968</v>
+      </c>
+      <c r="K94">
+        <f t="shared" si="2"/>
+        <v>0.11027813334728032</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>93</v>
       </c>
@@ -3088,8 +3312,20 @@
       <c r="G95">
         <v>3.64</v>
       </c>
-    </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I95">
+        <f t="shared" si="0"/>
+        <v>0.76919199999999999</v>
+      </c>
+      <c r="J95">
+        <f t="shared" si="1"/>
+        <v>0.87703591716645224</v>
+      </c>
+      <c r="K95">
+        <f t="shared" si="2"/>
+        <v>0.12296408283354776</v>
+      </c>
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>94</v>
       </c>
@@ -3111,8 +3347,20 @@
       <c r="G96">
         <v>3.36</v>
       </c>
-    </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I96">
+        <f t="shared" si="0"/>
+        <v>0.74608600000000003</v>
+      </c>
+      <c r="J96">
+        <f t="shared" si="1"/>
+        <v>0.86376269889362556</v>
+      </c>
+      <c r="K96">
+        <f t="shared" si="2"/>
+        <v>0.13623730110637444</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>95</v>
       </c>
@@ -3134,8 +3382,20 @@
       <c r="G97">
         <v>3.1</v>
       </c>
-    </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I97">
+        <f t="shared" si="0"/>
+        <v>0.72259800000000007</v>
+      </c>
+      <c r="J97">
+        <f t="shared" si="1"/>
+        <v>0.85005764510414239</v>
+      </c>
+      <c r="K97">
+        <f t="shared" si="2"/>
+        <v>0.14994235489585761</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>96</v>
       </c>
@@ -3157,8 +3417,20 @@
       <c r="G98">
         <v>2.87</v>
       </c>
-    </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I98">
+        <f t="shared" si="0"/>
+        <v>0.69911800000000002</v>
+      </c>
+      <c r="J98">
+        <f t="shared" si="1"/>
+        <v>0.83613276457749219</v>
+      </c>
+      <c r="K98">
+        <f t="shared" si="2"/>
+        <v>0.16386723542250781</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>97</v>
       </c>
@@ -3180,8 +3452,20 @@
       <c r="G99">
         <v>2.66</v>
       </c>
-    </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I99">
+        <f t="shared" si="0"/>
+        <v>0.675674</v>
+      </c>
+      <c r="J99">
+        <f t="shared" si="1"/>
+        <v>0.8219939172524332</v>
+      </c>
+      <c r="K99">
+        <f t="shared" si="2"/>
+        <v>0.1780060827475668</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>98</v>
       </c>
@@ -3203,8 +3487,20 @@
       <c r="G100">
         <v>2.4700000000000002</v>
       </c>
-    </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I100">
+        <f t="shared" si="0"/>
+        <v>0.65266800000000003</v>
+      </c>
+      <c r="J100">
+        <f t="shared" si="1"/>
+        <v>0.80787870376684645</v>
+      </c>
+      <c r="K100">
+        <f t="shared" si="2"/>
+        <v>0.19212129623315355</v>
+      </c>
+    </row>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>99</v>
       </c>
@@ -3226,8 +3522,20 @@
       <c r="G101">
         <v>2.2999999999999998</v>
       </c>
-    </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I101">
+        <f t="shared" si="0"/>
+        <v>0.63057000000000007</v>
+      </c>
+      <c r="J101">
+        <f t="shared" si="1"/>
+        <v>0.79408437838809054</v>
+      </c>
+      <c r="K101">
+        <f t="shared" si="2"/>
+        <v>0.20591562161190946</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>100</v>
       </c>
@@ -3249,8 +3557,20 @@
       <c r="G102">
         <v>2.14</v>
       </c>
-    </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I102">
+        <f t="shared" si="0"/>
+        <v>0.60807299999999997</v>
+      </c>
+      <c r="J102">
+        <f t="shared" si="1"/>
+        <v>0.77979035644203754</v>
+      </c>
+      <c r="K102">
+        <f t="shared" si="2"/>
+        <v>0.22020964355796246</v>
+      </c>
+    </row>
+    <row r="103" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>101</v>
       </c>
@@ -3272,8 +3592,20 @@
       <c r="G103">
         <v>2</v>
       </c>
-    </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I103">
+        <f t="shared" si="0"/>
+        <v>0.58527400000000007</v>
+      </c>
+      <c r="J103">
+        <f t="shared" si="1"/>
+        <v>0.76503202547344384</v>
+      </c>
+      <c r="K103">
+        <f t="shared" si="2"/>
+        <v>0.23496797452655616</v>
+      </c>
+    </row>
+    <row r="104" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>102</v>
       </c>
@@ -3295,8 +3627,20 @@
       <c r="G104">
         <v>1.87</v>
       </c>
-    </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I104">
+        <f t="shared" si="0"/>
+        <v>0.56227800000000006</v>
+      </c>
+      <c r="J104">
+        <f t="shared" si="1"/>
+        <v>0.74985198539445108</v>
+      </c>
+      <c r="K104">
+        <f t="shared" si="2"/>
+        <v>0.25014801460554892</v>
+      </c>
+    </row>
+    <row r="105" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>103</v>
       </c>
@@ -3318,8 +3662,20 @@
       <c r="G105">
         <v>1.75</v>
       </c>
-    </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I105">
+        <f t="shared" si="0"/>
+        <v>0.53920000000000001</v>
+      </c>
+      <c r="J105">
+        <f t="shared" si="1"/>
+        <v>0.73430239002743281</v>
+      </c>
+      <c r="K105">
+        <f t="shared" si="2"/>
+        <v>0.26569760997256719</v>
+      </c>
+    </row>
+    <row r="106" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>104</v>
       </c>
@@ -3341,8 +3697,20 @@
       <c r="G106">
         <v>1.63</v>
       </c>
-    </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I106">
+        <f t="shared" si="0"/>
+        <v>0.51615999999999995</v>
+      </c>
+      <c r="J106">
+        <f t="shared" si="1"/>
+        <v>0.71844276042006294</v>
+      </c>
+      <c r="K106">
+        <f t="shared" si="2"/>
+        <v>0.28155723957993706</v>
+      </c>
+    </row>
+    <row r="107" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>105</v>
       </c>
@@ -3364,8 +3732,20 @@
       <c r="G107">
         <v>1.52</v>
       </c>
-    </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I107">
+        <f t="shared" si="0"/>
+        <v>0.49196799999999996</v>
+      </c>
+      <c r="J107">
+        <f t="shared" si="1"/>
+        <v>0.70140430566114997</v>
+      </c>
+      <c r="K107">
+        <f t="shared" si="2"/>
+        <v>0.29859569433885003</v>
+      </c>
+    </row>
+    <row r="108" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A108">
         <v>106</v>
       </c>
@@ -3387,8 +3767,20 @@
       <c r="G108">
         <v>1.42</v>
       </c>
-    </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I108">
+        <f t="shared" si="0"/>
+        <v>0.46656600000000004</v>
+      </c>
+      <c r="J108">
+        <f t="shared" si="1"/>
+        <v>0.68305636663455527</v>
+      </c>
+      <c r="K108">
+        <f t="shared" si="2"/>
+        <v>0.31694363336544473</v>
+      </c>
+    </row>
+    <row r="109" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A109">
         <v>107</v>
       </c>
@@ -3410,8 +3802,20 @@
       <c r="G109">
         <v>1.32</v>
       </c>
-    </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I109">
+        <f t="shared" si="0"/>
+        <v>0.43989500000000004</v>
+      </c>
+      <c r="J109">
+        <f t="shared" si="1"/>
+        <v>0.66324580662074306</v>
+      </c>
+      <c r="K109">
+        <f t="shared" si="2"/>
+        <v>0.33675419337925694</v>
+      </c>
+    </row>
+    <row r="110" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A110">
         <v>108</v>
       </c>
@@ -3433,8 +3837,20 @@
       <c r="G110">
         <v>1.23</v>
       </c>
-    </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I110">
+        <f t="shared" si="0"/>
+        <v>0.41188899999999995</v>
+      </c>
+      <c r="J110">
+        <f t="shared" si="1"/>
+        <v>0.64178578980840639</v>
+      </c>
+      <c r="K110">
+        <f t="shared" si="2"/>
+        <v>0.35821421019159361</v>
+      </c>
+    </row>
+    <row r="111" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A111">
         <v>109</v>
       </c>
@@ -3456,8 +3872,20 @@
       <c r="G111">
         <v>1.1399999999999999</v>
       </c>
-    </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I111">
+        <f t="shared" si="0"/>
+        <v>0.38248400000000005</v>
+      </c>
+      <c r="J111">
+        <f t="shared" si="1"/>
+        <v>0.61845290847404055</v>
+      </c>
+      <c r="K111">
+        <f t="shared" si="2"/>
+        <v>0.38154709152595945</v>
+      </c>
+    </row>
+    <row r="112" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A112">
         <v>110</v>
       </c>
@@ -3479,8 +3907,20 @@
       <c r="G112">
         <v>1.05</v>
       </c>
-    </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I112">
+        <f t="shared" si="0"/>
+        <v>0.35160800000000003</v>
+      </c>
+      <c r="J112">
+        <f t="shared" si="1"/>
+        <v>0.59296542900914551</v>
+      </c>
+      <c r="K112">
+        <f t="shared" si="2"/>
+        <v>0.40703457099085449</v>
+      </c>
+    </row>
+    <row r="113" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A113">
         <v>111</v>
       </c>
@@ -3502,8 +3942,20 @@
       <c r="G113">
         <v>0.97</v>
       </c>
-    </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I113">
+        <f t="shared" si="0"/>
+        <v>0.31918800000000003</v>
+      </c>
+      <c r="J113">
+        <f t="shared" si="1"/>
+        <v>0.56496725568832751</v>
+      </c>
+      <c r="K113">
+        <f t="shared" si="2"/>
+        <v>0.43503274431167249</v>
+      </c>
+    </row>
+    <row r="114" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A114">
         <v>112</v>
       </c>
@@ -3525,8 +3977,20 @@
       <c r="G114">
         <v>0.89</v>
       </c>
-    </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I114">
+        <f t="shared" si="0"/>
+        <v>0.28514799999999996</v>
+      </c>
+      <c r="J114">
+        <f t="shared" si="1"/>
+        <v>0.53399250931075803</v>
+      </c>
+      <c r="K114">
+        <f t="shared" si="2"/>
+        <v>0.46600749068924197</v>
+      </c>
+    </row>
+    <row r="115" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A115">
         <v>113</v>
       </c>
@@ -3548,8 +4012,20 @@
       <c r="G115">
         <v>0.82</v>
       </c>
-    </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I115">
+        <f t="shared" si="0"/>
+        <v>0.24940499999999999</v>
+      </c>
+      <c r="J115">
+        <f t="shared" si="1"/>
+        <v>0.4994046455530825</v>
+      </c>
+      <c r="K115">
+        <f t="shared" si="2"/>
+        <v>0.5005953544469175</v>
+      </c>
+    </row>
+    <row r="116" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A116">
         <v>114</v>
       </c>
@@ -3571,8 +4047,20 @@
       <c r="G116">
         <v>0.75</v>
       </c>
-    </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I116">
+        <f t="shared" si="0"/>
+        <v>0.21187500000000004</v>
+      </c>
+      <c r="J116">
+        <f t="shared" si="1"/>
+        <v>0.46029881598804928</v>
+      </c>
+      <c r="K116">
+        <f t="shared" si="2"/>
+        <v>0.53970118401195077</v>
+      </c>
+    </row>
+    <row r="117" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A117">
         <v>115</v>
       </c>
@@ -3594,8 +4082,20 @@
       <c r="G117">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I117">
+        <f t="shared" si="0"/>
+        <v>0.17246899999999998</v>
+      </c>
+      <c r="J117">
+        <f t="shared" si="1"/>
+        <v>0.41529387185461814</v>
+      </c>
+      <c r="K117">
+        <f t="shared" si="2"/>
+        <v>0.58470612814538181</v>
+      </c>
+    </row>
+    <row r="118" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A118">
         <v>116</v>
       </c>
@@ -3617,8 +4117,20 @@
       <c r="G118">
         <v>0.64</v>
       </c>
-    </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I118">
+        <f t="shared" si="0"/>
+        <v>0.13109300000000002</v>
+      </c>
+      <c r="J118">
+        <f t="shared" si="1"/>
+        <v>0.36206767323250499</v>
+      </c>
+      <c r="K118">
+        <f t="shared" si="2"/>
+        <v>0.63793232676749501</v>
+      </c>
+    </row>
+    <row r="119" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A119">
         <v>117</v>
       </c>
@@ -3640,8 +4152,20 @@
       <c r="G119">
         <v>0.59</v>
       </c>
-    </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I119">
+        <f t="shared" si="0"/>
+        <v>8.764700000000003E-2</v>
+      </c>
+      <c r="J119">
+        <f t="shared" si="1"/>
+        <v>0.29605236023379383</v>
+      </c>
+      <c r="K119">
+        <f t="shared" si="2"/>
+        <v>0.70394763976620611</v>
+      </c>
+    </row>
+    <row r="120" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A120">
         <v>118</v>
       </c>
@@ -3663,8 +4187,20 @@
       <c r="G120">
         <v>0.54</v>
       </c>
-    </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I120">
+        <f t="shared" si="0"/>
+        <v>4.2030000000000012E-2</v>
+      </c>
+      <c r="J120">
+        <f t="shared" si="1"/>
+        <v>0.20501219475923868</v>
+      </c>
+      <c r="K120">
+        <f t="shared" si="2"/>
+        <v>0.79498780524076129</v>
+      </c>
+    </row>
+    <row r="121" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A121">
         <v>119</v>
       </c>
@@ -3685,9 +4221,803 @@
       </c>
       <c r="G121">
         <v>0.5</v>
+      </c>
+      <c r="I121">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J121">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="K121">
+        <f t="shared" si="2"/>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33DB695B-EB26-6043-85BA-8F071B0E499A}">
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="15.5" customWidth="1"/>
+    <col min="3" max="3" width="16.5" customWidth="1"/>
+    <col min="4" max="4" width="17.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>77</v>
+      </c>
+      <c r="B2">
+        <v>2.2882300000000001E-2</v>
+      </c>
+      <c r="C2">
+        <v>2.6983980000000001E-2</v>
+      </c>
+      <c r="D2">
+        <v>2.2882300000000001E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>77.5</v>
+      </c>
+      <c r="B3">
+        <v>2.2882300000000001E-2</v>
+      </c>
+      <c r="C3">
+        <v>2.806177E-2</v>
+      </c>
+      <c r="D3">
+        <v>2.2882300000000001E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>78</v>
+      </c>
+      <c r="B4">
+        <v>2.5214383E-2</v>
+      </c>
+      <c r="C4">
+        <v>2.918196E-2</v>
+      </c>
+      <c r="D4">
+        <v>2.5214380000000002E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>78.5</v>
+      </c>
+      <c r="B5">
+        <v>2.5214383E-2</v>
+      </c>
+      <c r="C5">
+        <v>3.0346169999999999E-2</v>
+      </c>
+      <c r="D5">
+        <v>2.5214380000000002E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>79</v>
+      </c>
+      <c r="B6">
+        <v>2.7769575000000001E-2</v>
+      </c>
+      <c r="C6">
+        <v>3.1556059999999997E-2</v>
+      </c>
+      <c r="D6">
+        <v>2.776957E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>79.5</v>
+      </c>
+      <c r="B7">
+        <v>2.7769575000000001E-2</v>
+      </c>
+      <c r="C7">
+        <v>3.2813370000000001E-2</v>
+      </c>
+      <c r="D7">
+        <v>2.776957E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>80</v>
+      </c>
+      <c r="B8">
+        <v>3.0804457E-2</v>
+      </c>
+      <c r="C8">
+        <v>3.4119879999999998E-2</v>
+      </c>
+      <c r="D8">
+        <v>3.0804459999999999E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>80.5</v>
+      </c>
+      <c r="B9">
+        <v>3.0804457E-2</v>
+      </c>
+      <c r="C9">
+        <v>3.5477460000000002E-2</v>
+      </c>
+      <c r="D9">
+        <v>3.0804459999999999E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>81</v>
+      </c>
+      <c r="B10">
+        <v>3.4094724999999999E-2</v>
+      </c>
+      <c r="C10">
+        <v>3.6888009999999999E-2</v>
+      </c>
+      <c r="D10">
+        <v>3.4094729999999997E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>81.5</v>
+      </c>
+      <c r="B11">
+        <v>3.4094724999999999E-2</v>
+      </c>
+      <c r="C11">
+        <v>3.8353520000000002E-2</v>
+      </c>
+      <c r="D11">
+        <v>3.4094729999999997E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>82</v>
+      </c>
+      <c r="B12">
+        <v>3.7710542999999999E-2</v>
+      </c>
+      <c r="C12">
+        <v>3.9876050000000003E-2</v>
+      </c>
+      <c r="D12">
+        <v>3.7710540000000001E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>82.5</v>
+      </c>
+      <c r="B13">
+        <v>3.7710542999999999E-2</v>
+      </c>
+      <c r="C13">
+        <v>4.14577E-2</v>
+      </c>
+      <c r="D13">
+        <v>3.7710540000000001E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>83</v>
+      </c>
+      <c r="B14">
+        <v>4.1739597000000003E-2</v>
+      </c>
+      <c r="C14">
+        <v>4.3100659999999999E-2</v>
+      </c>
+      <c r="D14">
+        <v>4.1739600000000002E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>83.5</v>
+      </c>
+      <c r="B15">
+        <v>4.1739597000000003E-2</v>
+      </c>
+      <c r="C15">
+        <v>4.4807199999999998E-2</v>
+      </c>
+      <c r="D15">
+        <v>4.1739600000000002E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>84</v>
+      </c>
+      <c r="B16">
+        <v>4.6300885999999999E-2</v>
+      </c>
+      <c r="C16">
+        <v>4.657965E-2</v>
+      </c>
+      <c r="D16">
+        <v>4.6300889999999997E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>84.5</v>
+      </c>
+      <c r="B17">
+        <v>4.6300885999999999E-2</v>
+      </c>
+      <c r="C17">
+        <v>4.8420419999999999E-2</v>
+      </c>
+      <c r="D17">
+        <v>4.6300889999999997E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>85</v>
+      </c>
+      <c r="B18">
+        <v>5.1593442000000003E-2</v>
+      </c>
+      <c r="C18">
+        <v>5.0332000000000002E-2</v>
+      </c>
+      <c r="D18">
+        <v>5.1593439999999997E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>85.5</v>
+      </c>
+      <c r="B19">
+        <v>5.1593442000000003E-2</v>
+      </c>
+      <c r="C19">
+        <v>5.2316950000000001E-2</v>
+      </c>
+      <c r="D19">
+        <v>5.1593439999999997E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>86</v>
+      </c>
+      <c r="B20">
+        <v>5.7552654000000002E-2</v>
+      </c>
+      <c r="C20">
+        <v>5.4377920000000003E-2</v>
+      </c>
+      <c r="D20">
+        <v>5.7552649999999997E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>86.5</v>
+      </c>
+      <c r="B21">
+        <v>5.7552654000000002E-2</v>
+      </c>
+      <c r="C21">
+        <v>5.6517629999999999E-2</v>
+      </c>
+      <c r="D21">
+        <v>5.7552649999999997E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>87</v>
+      </c>
+      <c r="B22">
+        <v>6.4315224000000004E-2</v>
+      </c>
+      <c r="C22">
+        <v>5.8738899999999997E-2</v>
+      </c>
+      <c r="D22">
+        <v>6.4315220000000006E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>87.5</v>
+      </c>
+      <c r="B23">
+        <v>6.4315224000000004E-2</v>
+      </c>
+      <c r="C23">
+        <v>6.1044599999999997E-2</v>
+      </c>
+      <c r="D23">
+        <v>6.4315220000000006E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>88</v>
+      </c>
+      <c r="B24">
+        <v>7.1774811999999993E-2</v>
+      </c>
+      <c r="C24">
+        <v>6.3437729999999998E-2</v>
+      </c>
+      <c r="D24">
+        <v>7.1774809999999994E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>88.5</v>
+      </c>
+      <c r="B25">
+        <v>7.1774811999999993E-2</v>
+      </c>
+      <c r="C25">
+        <v>6.5921350000000004E-2</v>
+      </c>
+      <c r="D25">
+        <v>7.1774809999999994E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>89</v>
+      </c>
+      <c r="B26">
+        <v>7.9786438000000001E-2</v>
+      </c>
+      <c r="C26">
+        <v>6.8498589999999998E-2</v>
+      </c>
+      <c r="D26">
+        <v>7.978644E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>89.5</v>
+      </c>
+      <c r="B27">
+        <v>7.9786438000000001E-2</v>
+      </c>
+      <c r="C27">
+        <v>7.117271E-2</v>
+      </c>
+      <c r="D27">
+        <v>7.978644E-2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>90</v>
+      </c>
+      <c r="B28">
+        <v>8.8794205000000001E-2</v>
+      </c>
+      <c r="C28">
+        <v>7.3947020000000002E-2</v>
+      </c>
+      <c r="D28">
+        <v>8.8794209999999998E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>90.5</v>
+      </c>
+      <c r="B29">
+        <v>8.8794205000000001E-2</v>
+      </c>
+      <c r="C29">
+        <v>7.6824939999999994E-2</v>
+      </c>
+      <c r="D29">
+        <v>8.8794209999999998E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>91</v>
+      </c>
+      <c r="B30">
+        <v>9.8869044000000003E-2</v>
+      </c>
+      <c r="C30">
+        <v>7.9809959999999999E-2</v>
+      </c>
+      <c r="D30">
+        <v>9.8869040000000005E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>91.5</v>
+      </c>
+      <c r="B31">
+        <v>9.8869044000000003E-2</v>
+      </c>
+      <c r="C31">
+        <v>8.2905679999999995E-2</v>
+      </c>
+      <c r="D31">
+        <v>9.8869040000000005E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32">
+        <v>92</v>
+      </c>
+      <c r="B32">
+        <v>0.110278133</v>
+      </c>
+      <c r="C32">
+        <v>8.6115769999999994E-2</v>
+      </c>
+      <c r="D32">
+        <v>0.11027813</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33">
+        <v>92.5</v>
+      </c>
+      <c r="B33">
+        <v>0.110278133</v>
+      </c>
+      <c r="C33">
+        <v>8.9443990000000001E-2</v>
+      </c>
+      <c r="D33">
+        <v>0.11027813</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34">
+        <v>93</v>
+      </c>
+      <c r="B34">
+        <v>0.122964083</v>
+      </c>
+      <c r="C34">
+        <v>9.2894180000000007E-2</v>
+      </c>
+      <c r="D34">
+        <v>0.12296408</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35">
+        <v>93.5</v>
+      </c>
+      <c r="B35">
+        <v>0.122964083</v>
+      </c>
+      <c r="C35">
+        <v>9.647029E-2</v>
+      </c>
+      <c r="D35">
+        <v>0.12296408</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36">
+        <v>94</v>
+      </c>
+      <c r="B36">
+        <v>0.13623730100000001</v>
+      </c>
+      <c r="C36">
+        <v>0.10017631</v>
+      </c>
+      <c r="D36">
+        <v>0.13623730000000001</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A37">
+        <v>94.5</v>
+      </c>
+      <c r="B37">
+        <v>0.13623730100000001</v>
+      </c>
+      <c r="C37">
+        <v>0.10401636</v>
+      </c>
+      <c r="D37">
+        <v>0.13623730000000001</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38">
+        <v>95</v>
+      </c>
+      <c r="B38">
+        <v>0.149942355</v>
+      </c>
+      <c r="C38">
+        <v>0.10799458000000001</v>
+      </c>
+      <c r="D38">
+        <v>0.14994235</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39">
+        <v>95.5</v>
+      </c>
+      <c r="B39">
+        <v>0.149942355</v>
+      </c>
+      <c r="C39">
+        <v>0.11211524</v>
+      </c>
+      <c r="D39">
+        <v>0.14994235</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A40">
+        <v>96</v>
+      </c>
+      <c r="B40">
+        <v>0.163867235</v>
+      </c>
+      <c r="C40">
+        <v>0.11638264</v>
+      </c>
+      <c r="D40">
+        <v>0.16386724</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A41">
+        <v>96.5</v>
+      </c>
+      <c r="B41">
+        <v>0.163867235</v>
+      </c>
+      <c r="C41">
+        <v>0.12080117</v>
+      </c>
+      <c r="D41">
+        <v>0.16386724</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A42">
+        <v>97</v>
+      </c>
+      <c r="B42">
+        <v>0.17800608300000001</v>
+      </c>
+      <c r="C42">
+        <v>0.12537525999999999</v>
+      </c>
+      <c r="D42">
+        <v>0.17800608000000001</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A43">
+        <v>97.5</v>
+      </c>
+      <c r="B43">
+        <v>0.17800608300000001</v>
+      </c>
+      <c r="C43">
+        <v>0.13010941000000001</v>
+      </c>
+      <c r="D43">
+        <v>0.17800608000000001</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A44">
+        <v>98</v>
+      </c>
+      <c r="B44">
+        <v>0.192121296</v>
+      </c>
+      <c r="C44">
+        <v>0.13500817000000001</v>
+      </c>
+      <c r="D44">
+        <v>0.19212129999999999</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A45">
+        <v>98.5</v>
+      </c>
+      <c r="B45">
+        <v>0.192121296</v>
+      </c>
+      <c r="C45">
+        <v>0.14007612</v>
+      </c>
+      <c r="D45">
+        <v>0.19212129999999999</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A46">
+        <v>99</v>
+      </c>
+      <c r="B46">
+        <v>0.20591562199999999</v>
+      </c>
+      <c r="C46">
+        <v>0.14531789000000001</v>
+      </c>
+      <c r="D46">
+        <v>0.20591561999999999</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47">
+        <v>99.5</v>
+      </c>
+      <c r="B47">
+        <v>0.20591562199999999</v>
+      </c>
+      <c r="C47">
+        <v>0.15073810000000001</v>
+      </c>
+      <c r="D47">
+        <v>0.20591561999999999</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A48">
+        <v>100</v>
+      </c>
+      <c r="B48">
+        <v>0.22020964400000001</v>
+      </c>
+      <c r="C48">
+        <v>0.15634144</v>
+      </c>
+      <c r="D48">
+        <v>0.22020964000000001</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49">
+        <v>100.5</v>
+      </c>
+      <c r="B49">
+        <v>0.22020964400000001</v>
+      </c>
+      <c r="C49">
+        <v>0.16213254999999999</v>
+      </c>
+      <c r="D49">
+        <v>0.22020964000000001</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50">
+        <v>101</v>
+      </c>
+      <c r="B50">
+        <v>0.234967975</v>
+      </c>
+      <c r="C50">
+        <v>0.16811609</v>
+      </c>
+      <c r="D50">
+        <v>0.23496797</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51">
+        <v>101.5</v>
+      </c>
+      <c r="B51">
+        <v>0.234967975</v>
+      </c>
+      <c r="C51">
+        <v>0.1</v>
+      </c>
+      <c r="D51">
+        <v>0.23496797</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52">
+        <v>102</v>
+      </c>
+      <c r="B52">
+        <v>0.250148015</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53">
+        <v>102.5</v>
+      </c>
+      <c r="B53">
+        <v>0.250148015</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54">
+        <v>103</v>
+      </c>
+      <c r="B54">
+        <v>0.26569760999999997</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55">
+        <v>103.5</v>
+      </c>
+      <c r="B55">
+        <v>0.26569760999999997</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A56">
+        <v>104</v>
+      </c>
+      <c r="B56">
+        <v>0.28155723999999999</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A57">
+        <v>104.5</v>
+      </c>
+      <c r="B57">
+        <v>0.28155723999999999</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A58">
+        <v>105</v>
+      </c>
+      <c r="B58">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Validation complete against the excel model
</commit_message>
<xml_diff>
--- a/2022 Actuarial Life Table.xlsx
+++ b/2022 Actuarial Life Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sodamkim/Library/CloudStorage/Box-Box/ATTR-CM_SK/CEA/Microsimulation/Dark Peak Analytics/TRACE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6064FC80-04DB-C444-9D3D-5D7B97B6BFF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9950EE3-D5BC-C24E-A634-F80E33BB74C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22380" yWindow="4000" windowWidth="28040" windowHeight="17180" activeTab="1" xr2:uid="{49FD46BD-3C6D-9D48-A728-0523D1ADC09C}"/>
+    <workbookView xWindow="1500" yWindow="3260" windowWidth="28040" windowHeight="17180" xr2:uid="{49FD46BD-3C6D-9D48-A728-0523D1ADC09C}"/>
   </bookViews>
   <sheets>
     <sheet name="2022 Actuarial Life Table" sheetId="1" r:id="rId1"/>

</xml_diff>